<commit_message>
stand flow and item import refactor
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/Contact.xlsx
+++ b/src/test/resources/testData/Contact.xlsx
@@ -12,11 +12,32 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="24">
   <si>
     <t>SKU</t>
   </si>
   <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Family</t>
+  </si>
+  <si>
+    <t>isTestEvent</t>
+  </si>
+  <si>
+    <t>NewBoolean</t>
+  </si>
+  <si>
+    <t>NewText</t>
+  </si>
+  <si>
+    <t>NewSelect</t>
+  </si>
+  <si>
+    <t>NewDate</t>
+  </si>
+  <si>
     <t>DIA_FirstName</t>
   </si>
   <si>
@@ -32,10 +53,37 @@
     <t>İsim</t>
   </si>
   <si>
-    <t>Kişi-10</t>
-  </si>
-  <si>
-    <t>28cedb21-7210-4c1b-9396-6c844a923bdf</t>
+    <t>0e43d2e8-ffd3-425a-b27a-0fc3a61d47d3</t>
+  </si>
+  <si>
+    <t>IWSA</t>
+  </si>
+  <si>
+    <t>b33a2b43-8c07-4d5a-8087-d93cc0ee39c9</t>
+  </si>
+  <si>
+    <t>Reserve</t>
+  </si>
+  <si>
+    <t>ffe5799a-e160-4723-8e6d-62172323661f</t>
+  </si>
+  <si>
+    <t>0f54952b-7903-46c4-94bc-ae29c8cb440a</t>
+  </si>
+  <si>
+    <t>3289f35d-b677-40e2-ab89-6c20c7452089</t>
+  </si>
+  <si>
+    <t>Kişi-05</t>
+  </si>
+  <si>
+    <t>9018e1b0-b93c-43e3-95b0-2bb72ad9b2f8</t>
+  </si>
+  <si>
+    <t>5498381895</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
@@ -80,7 +128,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -88,7 +136,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s" s="0">
         <v>2</v>
@@ -99,13 +147,94 @@
       <c r="E1" t="s" s="0">
         <v>4</v>
       </c>
+      <c r="F1" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="J1" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s" s="0">
+        <v>11</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s" s="0">
-        <v>7</v>
+        <v>13</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="I4" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="I5" t="s" s="0">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="I6" t="s" s="0">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="I7" t="s" s="0">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="I9" t="s" s="0">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
locate and resource update
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/Contact.xlsx
+++ b/src/test/resources/testData/Contact.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="25">
   <si>
     <t>SKU</t>
   </si>
@@ -56,16 +56,37 @@
     <t>İsim</t>
   </si>
   <si>
-    <t>Kişi-12</t>
-  </si>
-  <si>
-    <t>30d226f4-6e81-455c-8e21-9518be943212</t>
-  </si>
-  <si>
-    <t>Kişi-18</t>
-  </si>
-  <si>
-    <t>xxx</t>
+    <t>e6bc1217-db31-42d4-b8be-725d12fb9aa6</t>
+  </si>
+  <si>
+    <t>IWSA</t>
+  </si>
+  <si>
+    <t>dc85684e-8a2e-4638-a8a9-a4402d198278</t>
+  </si>
+  <si>
+    <t>Reserve</t>
+  </si>
+  <si>
+    <t>f395e115-8338-4ae5-a15e-984f97ce0aee</t>
+  </si>
+  <si>
+    <t>de912498-d25d-4bf3-85b0-931ae12391cc</t>
+  </si>
+  <si>
+    <t>a2ff5b6b-b3f1-4c5d-a9da-7da2a2632cf7</t>
+  </si>
+  <si>
+    <t>Kişi-01</t>
+  </si>
+  <si>
+    <t>07a72fc2-a9fc-4ac1-a486-13916ccd89ab</t>
+  </si>
+  <si>
+    <t>Kişi-10</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
@@ -110,7 +131,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -158,7 +179,7 @@
       <c r="A2" t="s" s="0">
         <v>14</v>
       </c>
-      <c r="I2" t="s" s="0">
+      <c r="C2" t="s" s="0">
         <v>15</v>
       </c>
     </row>
@@ -166,11 +187,60 @@
       <c r="A3" t="s" s="0">
         <v>16</v>
       </c>
-      <c r="I3" t="s" s="0">
-        <v>15</v>
-      </c>
-      <c r="M3" t="s" s="0">
-        <v>17</v>
+      <c r="B3" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="I4" t="s" s="0">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="I5" t="s" s="0">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="I6" t="s" s="0">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="I7" t="s" s="0">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="I9" t="s" s="0">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>